<commit_message>
Implement prompt 18 technical execution
</commit_message>
<xml_diff>
--- a/data/excel/checklists.xlsx
+++ b/data/excel/checklists.xlsx
@@ -26,6 +26,24 @@
   </x:si>
   <x:si>
     <x:t>Items</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TipoOT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FamiliaActivo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PlanPreventivoCodigo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CodigoTarea</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ActivoCodigo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Activo</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -398,9 +416,15 @@
     <x:col min="2" max="2" width="8.282054" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="4.710625" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="5.853482" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="7.424911" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12.853482" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20.853482" style="0" customWidth="1"/>
+    <x:col min="8" max="8" width="11.996339" style="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12.853482" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="6.282054" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:4">
+    <x:row r="1" spans="1:10">
       <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -412,6 +436,24 @@
       </x:c>
       <x:c r="D1" s="1" t="s">
         <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1" s="1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F1" s="1" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G1" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H1" s="1" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="I1" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J1" s="1" t="s">
+        <x:v>9</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>